<commit_message>
Mapping Document review fixes: text cells, row-aligned diff, per-field winners (ticket 11)
Three-axis review:
- Every generated cell is text, so a number or date reads back the same;
  text starting with "=" stays text, never a formula.
- `diff` aligns rows by content: one row added is one line, not every row
  below it; row numbers are the spreadsheet's.
- `--only` selects by source or kind name, not by folder name.
- The identifiers that join records come from activation.NAMESPACES.
- "Who wins" per MDM field (source and kind), conditions and quality tests
  in plain words (a test holds every name covered), and every exception
  check listed as a critical data element.
- A workbook regenerated from unchanged rules is the same bytes (fixed zip
  entry times and modified stamp); *.xlsx is binary to git.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V75sGum1vG9w3NFXJLh4XQ
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kind" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preferred sources" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matching rules" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Who wins each field" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classification" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matching rules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -574,6 +575,466 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MDM field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Filled by, first wins</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Rules path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1, gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>fiscal_year_end</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>gleif_entity_creation_date</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>gleif_entity_status</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>gleif_initial_registration</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>gleif_last_update</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>gleif_legal_form</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>gleif_managing_lou</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>gleif_next_renewal</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>gleif_registration_authority</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>gleif_registration_authority_entity_id</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>gleif_registration_status</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>gleif_validation_source</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>jurisdiction</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1, gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>sic</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>sic_description</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>state_of_incorporation</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -658,7 +1119,7 @@
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: sic; values: 6189)</t>
+          <t>sic is one of: 6189</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -700,7 +1161,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: sic; values: 6221)</t>
+          <t>sic is one of: 6221</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -742,7 +1203,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: sic; values: 8888)</t>
+          <t>sic is one of: 8888</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -784,7 +1245,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>fields_all_empty@1(fields: ticker); token_match@2(field: category; normalizer: conformed; token_list: emerging_growth; min_count: 1)</t>
+          <t>ticker is empty; and category holds at least 1 word(s) of the list emerging_growth</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -826,7 +1287,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: operating); token_match@2(field: entity_name; normalizer: conformed; token_list: fund_name; min_count: 1)</t>
+          <t>entity_type is one of: operating; and entity_name holds at least 1 word(s) of the list fund_name</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -868,7 +1329,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: operating); field_in_set@1(field: sic; values: 6199, 6211, 6282, 6799, 6798); field_in_set@1(field: category; values: &lt;br&gt;Emerging growth company)</t>
+          <t>entity_type is one of: operating; and sic is one of: 6199, 6211, 6282, 6799, 6798; and category is one of: &lt;br&gt;Emerging growth company</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -910,7 +1371,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: operating); field_in_set@1(field: sic; values: 6798); fields_all_empty@1(fields: ticker)</t>
+          <t>entity_type is one of: operating; and sic is one of: 6798; and ticker is empty</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -948,7 +1409,7 @@
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: operating); fields_all_empty@1(fields: industry_code)</t>
+          <t>entity_type is one of: operating; and industry_code is empty</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -990,7 +1451,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: operating); values_overlap@1(field: forms; values: fund_report; min_count: 1)</t>
+          <t>entity_type is one of: operating; and forms holds at least 1 of the list fund_report</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1032,7 +1493,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: operating); values_overlap@1(field: forms; values: form_10; min_count: 1); values_overlap@1(field: forms; values: private_offering; min_count: 1); values_overlap@1(field: forms; values: bdc_election; max_count: 0)</t>
+          <t>entity_type is one of: operating; and forms holds at least 1 of the list form_10; and forms holds at least 1 of the list private_offering; and forms holds at least  of the list bdc_election</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1070,7 +1531,7 @@
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: operating)</t>
+          <t>entity_type is one of: operating</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1112,7 +1573,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: other); token_match@2(field: entity_name; normalizer: conformed; token_list: person_suffix; min_count: 1)</t>
+          <t>entity_type is one of: other; and entity_name holds at least 1 word(s) of the list person_suffix</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1150,7 +1611,7 @@
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>field_in_set@1(field: entity_type; values: other); evidence_present@1(document: sic); evidence_present@1(document: category); token_match@2(field: entity_name; normalizer: conformed; token_list: company_legal_form; min_count: 1)</t>
+          <t>entity_type is one of: other; and The record has sic; and The record has category; and entity_name holds at least 1 word(s) of the list company_legal_form</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1188,7 +1649,7 @@
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>otherwise</t>
+          <t>Otherwise</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1202,7 +1663,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1291,7 +1752,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>name_census_match@1(sec_normalizer: normalize_text@sec-legal-form-kept-v1; gleif_normalizer: normalize_text@legal-form-kept-v1); gleif_entity_eligible@1(categories: GENERAL; entity_statuses: ACTIVE; refused_registration_statuses: ANNULLED, DUPLICATE); holds_no_other_lei@1(); jurisdiction_agrees@1(sec_field: state_of_incorporation; sec_codes: edgar-iso-v1; gleif_field: jurisdiction)</t>
+          <t>The names are equal, legal form kept, and exactly one SEC filer and one GLEIF entity carry that name; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI; and SEC's state_of_incorporation names the same place as GLEIF's jurisdiction</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1333,7 +1794,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>name_census_match@1(sec_normalizer: normalize_text@sec-legal-form-kept-v1; gleif_normalizer: normalize_text@legal-form-kept-v1); gleif_entity_eligible@1(categories: GENERAL; entity_statuses: ACTIVE; refused_registration_statuses: ANNULLED, DUPLICATE); holds_no_other_lei@1(); jurisdictions_do_not_conflict@1(sec_field: state_of_incorporation; sec_codes: edgar-iso-v1; gleif_field: jurisdiction; sec_business_country: matching.business_country); postal_agrees@1(sec_code: matching.business_postal_code; sec_country: matching.business_country; gleif_code: matching.headquarters_postal_code; gleif_country: matching.headquarters_country)</t>
+          <t>The names are equal, legal form kept, and exactly one SEC filer and one GLEIF entity carry that name; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI; and SEC's state_of_incorporation and GLEIF's jurisdiction do not name different places; and SEC's business postcode equals GLEIF's headquarters postcode, in the same country</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -1352,7 +1813,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1405,7 +1866,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1423,7 +1884,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
A winner for one field: the Mapping Document shows it; the skill writes it (rules skill ticket 12)
PR #743 said one field's winner "can't be set on its own". Wrong: the merge
engine takes a rule per field, `kinds.<kind>.fields.<name>`, which inherits
`defaults` and may change any part of it, its source order included
(survivorship._select_values).

- "Who wins" (source and kind workbooks) reads each field's rule as the
  engine does: its own when it has one, else the kind's default, and says
  which.
- The Rules skill turns a steward's per-field winner into
  `fields.<name>.sources`, approved by that steward; REFERENCE.md names
  what a field's own rule may change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V75sGum1vG9w3NFXJLh4XQ
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -575,13 +575,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="43" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -602,6 +603,11 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Rules path</t>
         </is>
       </c>
@@ -624,6 +630,11 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -646,6 +657,11 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -668,6 +684,11 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -690,6 +711,11 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -712,6 +738,11 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -734,6 +765,11 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -756,6 +792,11 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -778,6 +819,11 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -800,6 +846,11 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -822,6 +873,11 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -844,6 +900,11 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -866,6 +927,11 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -888,6 +954,11 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -910,6 +981,11 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -932,6 +1008,11 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -954,6 +1035,11 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -976,6 +1062,11 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -998,6 +1089,11 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>
       </c>
@@ -1019,6 +1115,11 @@
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Kind default</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>

</xml_diff>

<commit_message>
Profiling 07: ADV rules (switched off), pinned tests, and the closure blocker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01FFKdv4nqKXKM9d5Cf2hEFk
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -578,6 +578,40 @@
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/company.yaml defaults.sources[2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>iapd.adv.filings.v1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources[3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>iapd.adv.custody.v1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources[4]</t>
         </is>
       </c>
     </row>
@@ -596,7 +630,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="43" customWidth="1" min="5" max="5"/>
@@ -637,7 +671,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>sec.submissions.company.v1, gleif.level1.v1</t>
+          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custody.v1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1042,7 +1076,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>sec.submissions.company.v1, gleif.level1.v1</t>
+          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custody.v1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1787,7 +1821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2255,6 +2289,120 @@
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/company.yaml rules[10]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>iapd-adv-crd</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09.1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>iapd.adv.filings.v1</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>The record's CRD is the one a Company holds; and Exactly one Company holds that CRD, or none</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml rules[11]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>iapd-adv-custodian-lei</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09.1</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>iapd.adv.custody.v1</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml rules[12]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>iapd-adv-custodian-bd</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09.1</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>iapd.adv.custody.v1</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>The record's BD_NUMBER is the one a Company holds; and Exactly one Company holds that BD_NUMBER, or none</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml rules[13]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Profiling 07: custodians one record per file, no MDM link; smoke run
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_01FFKdv4nqKXKM9d5Cf2hEFk
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.custody.v1</t>
+          <t>iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custody.v1</t>
+          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custody.v1</t>
+          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.custody.v1</t>
+          <t>iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.custody.v1</t>
+          <t>iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
N-PORT registrant as a Company (ticket 79, part 2): configuration and test run
Reads N-PORT's registrant and submission tables, keeps each CIK's latest
filing whole, and maps it to a Company by CIK (sec.nport.registrant.v1),
with the SEC file number and stated LEI lookup only. The Company rules gain
nport-registrant-cik (creates when none holds the CIK; operator "agreed"),
declared, not switched on. Mapping Documents regenerated. Test run: 1,947
registrants accepted, none set aside.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XffcaJSmoXmrPyZxCeFHRa
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -612,6 +612,23 @@
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/company.yaml defaults.sources[4]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.registrant.v1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml defaults.sources[5]</t>
         </is>
       </c>
     </row>
@@ -671,7 +688,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custodians.v1</t>
+          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custodians.v1, sec.nport.registrant.v1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1076,7 +1093,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custodians.v1</t>
+          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custodians.v1, sec.nport.registrant.v1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1821,7 +1838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1922,32 +1939,28 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-name-jurisdiction</t>
+          <t>nport-registrant-cik</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25.1</t>
+          <t>2026-10-15.1</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
+          <t>sec.nport.registrant.v1</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>The names are equal, legal form kept, and exactly one SEC filer and one GLEIF entity carry that name; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI; and SEC's state_of_incorporation names the same place as GLEIF's jurisdiction</t>
+          <t>The record's CIK is the one a Company holds; and Exactly one Company holds that CIK, or none</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>mint</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1964,12 +1977,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-name-postal</t>
+          <t>sec-gleif-name-jurisdiction</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25.2</t>
+          <t>2026-09-25.1</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1984,7 +1997,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>The names are equal, legal form kept, and exactly one SEC filer and one GLEIF entity carry that name; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI; and SEC's state_of_incorporation and GLEIF's jurisdiction do not name different places; and SEC's business postcode equals GLEIF's headquarters postcode, in the same country</t>
+          <t>The names are equal, legal form kept, and exactly one SEC filer and one GLEIF entity carry that name; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI; and SEC's state_of_incorporation names the same place as GLEIF's jurisdiction</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -2006,12 +2019,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p1</t>
+          <t>sec-gleif-name-postal</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28.1</t>
+          <t>2026-09-25.2</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2026,7 +2039,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Pass P1: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>The names are equal, legal form kept, and exactly one SEC filer and one GLEIF entity carry that name; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI; and SEC's state_of_incorporation and GLEIF's jurisdiction do not name different places; and SEC's business postcode equals GLEIF's headquarters postcode, in the same country</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -2048,7 +2061,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p2</t>
+          <t>sec-gleif-cascade-p1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -2068,7 +2081,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Pass P2: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P1: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2090,7 +2103,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p3</t>
+          <t>sec-gleif-cascade-p2</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2110,7 +2123,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Pass P3: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P2: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2132,7 +2145,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p4</t>
+          <t>sec-gleif-cascade-p3</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2152,7 +2165,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P3: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2174,7 +2187,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p5</t>
+          <t>sec-gleif-cascade-p4</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2194,7 +2207,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2216,7 +2229,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p6</t>
+          <t>sec-gleif-cascade-p5</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2236,7 +2249,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2258,7 +2271,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p7</t>
+          <t>sec-gleif-cascade-p6</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2278,7 +2291,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2300,28 +2313,32 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>iapd-adv-crd</t>
+          <t>sec-gleif-cascade-p7</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09.1</t>
+          <t>2026-09-28.1</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.filings.v1</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>sec.submissions.company.v1</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>The record's CRD is the one a Company holds; and Exactly one Company holds that CRD, or none</t>
+          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>mint</t>
+          <t>wait</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -2338,7 +2355,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>iapd-adv-custodian-lei</t>
+          <t>iapd-adv-crd</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2348,13 +2365,13 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.custodians.v1</t>
+          <t>iapd.adv.filings.v1</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
+          <t>The record's CRD is the one a Company holds; and Exactly one Company holds that CRD, or none</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -2376,7 +2393,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>iapd-adv-custodian-bd</t>
+          <t>iapd-adv-custodian-lei</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -2392,17 +2409,55 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml rules[13]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>iapd-adv-custodian-bd</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09.1</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>iapd.adv.custodians.v1</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>The record's BD_NUMBER is the one a Company holds; and Exactly one Company holds that BD_NUMBER, or none</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>mint</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/company.yaml rules[13]</t>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml rules[14]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 16, item 10: a kind's Mapping Document names its own kind
The identifier condition words said "a Company holds" for every kind, and a
condition with only a ceiling (max_count: 0) read "at least  of the list".
Each kind now names itself, and the count reads as a floor, a ceiling, both,
or "none". The three kind workbooks are regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -1414,7 +1414,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>ticker is empty; and category holds at least 1 word(s) of the list emerging_growth</t>
+          <t>ticker is empty; and category holds at least 1 of the words of the list emerging_growth</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>entity_type is one of: operating; and entity_name holds at least 1 word(s) of the list fund_name</t>
+          <t>entity_type is one of: operating; and entity_name holds at least 1 of the words of the list fund_name</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>entity_type is one of: operating; and forms holds at least 1 of the list form_10; and forms holds at least 1 of the list private_offering; and forms holds at least  of the list bdc_election</t>
+          <t>entity_type is one of: operating; and forms holds at least 1 of the list form_10; and forms holds at least 1 of the list private_offering; and forms holds none of the list bdc_election</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>entity_type is one of: other; and entity_name holds at least 1 word(s) of the list person_suffix</t>
+          <t>entity_type is one of: other; and entity_name holds at least 1 of the words of the list person_suffix</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1780,7 +1780,7 @@
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>entity_type is one of: other; and The record has sic; and The record has category; and entity_name holds at least 1 word(s) of the list company_legal_form</t>
+          <t>entity_type is one of: other; and The record has sic; and The record has category; and entity_name holds at least 1 of the words of the list company_legal_form</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ticket 16, item 10: review fixes to the count and pass words
A floor of 0 is no floor ("at most 2"), equal bounds read "exactly 1", and
a cascade pass with no refused flags says "none" instead of an empty list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -2081,7 +2081,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Pass P1: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P1: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Pass P2: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P2: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Pass P3: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P3: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ticket 16, item 10: a kind's Mapping Document names its own kind (#1009)
* Ticket 16, item 10: a kind's Mapping Document names its own kind

The identifier condition words said "a Company holds" for every kind, and a
condition with only a ceiling (max_count: 0) read "at least  of the list".
Each kind now names itself, and the count reads as a floor, a ceiling, both,
or "none". The three kind workbooks are regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

* Ticket 16, item 10: review fixes to the count and pass words

A floor of 0 is no floor ("at most 2"), equal bounds read "exactly 1", and
a cascade pass with no refused flags says "none" instead of an empty list.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Aneena Ananth <aneenaananth@MacBook-Pro.local>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -1414,7 +1414,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>ticker is empty; and category holds at least 1 word(s) of the list emerging_growth</t>
+          <t>ticker is empty; and category holds at least 1 of the words of the list emerging_growth</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>entity_type is one of: operating; and entity_name holds at least 1 word(s) of the list fund_name</t>
+          <t>entity_type is one of: operating; and entity_name holds at least 1 of the words of the list fund_name</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>entity_type is one of: operating; and forms holds at least 1 of the list form_10; and forms holds at least 1 of the list private_offering; and forms holds at least  of the list bdc_election</t>
+          <t>entity_type is one of: operating; and forms holds at least 1 of the list form_10; and forms holds at least 1 of the list private_offering; and forms holds none of the list bdc_election</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>entity_type is one of: other; and entity_name holds at least 1 word(s) of the list person_suffix</t>
+          <t>entity_type is one of: other; and entity_name holds at least 1 of the words of the list person_suffix</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1780,7 +1780,7 @@
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>entity_type is one of: other; and The record has sic; and The record has category; and entity_name holds at least 1 word(s) of the list company_legal_form</t>
+          <t>entity_type is one of: other; and The record has sic; and The record has category; and entity_name holds at least 1 of the words of the list company_legal_form</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Pass P1: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P1: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Pass P2: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P2: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Pass P3: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P3: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: ; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ticket 97: a GLEIF issuer record creates or joins its Company by LEI
- mdm.prepare: optional record_extras copies named row columns into the
  record (record_column); absent or null adds nothing; a clash is refused.
- Binding rules may carry record tests (classification family) that narrow
  the records they apply to; they read the record alone.
- GLEIF Level 1 reading: an nport_issuers reference flags the LEIs an N-PORT
  holding names as issuer; the Level 1 contract adds matching.nport_issuer on
  top of its unchanged matching values (base), so a record without the flag
  reads exactly as before (assertion ids unchanged).
- company.yaml: rule gleif-issuer-lei (declared, not switched on), and GLEIF
  as an LEI source; policy and contract digest layers added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -1838,7 +1838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2458,6 +2458,44 @@
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/company.yaml rules[14]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>gleif-issuer-lei</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16.1</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>The record has provenance.matching.nport_issuer; and The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>mint</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>merge/kinds/company.yaml rules[15]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 22: the issuer rule joins and waits, never creates
The operator ruled configuration only ("Wait, config only"): gleif-issuer-lei
version 2026-10-16.2 sets on_no_match: wait, so an issuer joins the one
Company holding its LEI and otherwise waits for the SEC-GLEIF name rules.
Proving Run 2 had 3,240 issuers that are SEC filers become a second Company.
Ticket 99 (an engine change) closed, replaced. Tests: an issuer no Company
holds creates nothing (fails with mint); an issuer joins the Company an ADV
custodian gave the LEI. Pinned digests: only the top Company layer and the
whole policy move. Mapping Documents regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199JiQoZJ5my5vrS5tW3FQH
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -2474,7 +2474,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16.1</t>
+          <t>2026-10-16.2</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>mint</t>
+          <t>wait</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Ticket 09: delete cascade passes P2 and P3
The operator's ruling (2026-10-17): "Delete both (Recommended)". P2 (street
and postcode) gives 8 new links and P3 (street and city) 22, below the 52 a
pass needs to be proved. A pair either matched shares the postcode (P4) or
the city (P5). The other passes keep their names.

Company's policy digests move by one layer (without_p2_p3_deleted: peeled,
the policy is the one before); the Mapping Document is regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199JiQoZJ5my5vrS5tW3FQH
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -1838,7 +1838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p2</t>
+          <t>sec-gleif-cascade-p4</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Pass P2: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p3</t>
+          <t>sec-gleif-cascade-p5</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Pass P3: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p4</t>
+          <t>sec-gleif-cascade-p6</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p5</t>
+          <t>sec-gleif-cascade-p7</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2271,32 +2271,28 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p6</t>
+          <t>iapd-adv-crd</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28.1</t>
+          <t>2026-10-09.1</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
+          <t>iapd.adv.filings.v1</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>The record's CRD is the one a Company holds; and Exactly one Company holds that CRD, or none</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>mint</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -2313,32 +2309,28 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p7</t>
+          <t>iapd-adv-custodian-lei</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28.1</t>
+          <t>2026-10-09.1</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
+          <t>iapd.adv.custodians.v1</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>mint</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -2355,7 +2347,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>iapd-adv-crd</t>
+          <t>iapd-adv-custodian-bd</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -2365,13 +2357,13 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.filings.v1</t>
+          <t>iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>The record's CRD is the one a Company holds; and Exactly one Company holds that CRD, or none</t>
+          <t>The record's BD_NUMBER is the one a Company holds; and Exactly one Company holds that BD_NUMBER, or none</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -2393,109 +2385,33 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>iapd-adv-custodian-lei</t>
+          <t>gleif-issuer-lei</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09.1</t>
+          <t>2026-10-16.2</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.custodians.v1</t>
+          <t>gleif.level1.v1</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
+          <t>The record has provenance.matching.nport_issuer; and The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>mint</t>
+          <t>wait</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/company.yaml rules[13]</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>iapd-adv-custodian-bd</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09.1</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>iapd.adv.custodians.v1</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>The record's BD_NUMBER is the one a Company holds; and Exactly one Company holds that BD_NUMBER, or none</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>mint</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/company.yaml rules[14]</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>gleif-issuer-lei</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-16.2</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>gleif.level1.v1</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>The record has provenance.matching.nport_issuer; and The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>wait</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/company.yaml rules[15]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 129, fixes 2 and 3: GLEIF's dates and the SIC label leave the Company
GLEIF's LastUpdateDate and NextRenewalDate are no longer Company fields; the
census matching rules (record_pairs.rs) check that the census saw the GLEIF
version the Stage holds by its effective time, compared as an instant with
GLEIF's own spelling. sic_description leaves the Company's Dataset Contract
(RDM sec-sic-codes holds the labels; silver keeps the filed one). Migration 026
recreates the Company writer without the three columns and drops them.

Digest tests gain one layer each (with the fields put back, every contract and
the cohort is the one pinned before); a populated-store test for 026; the
mapping workbooks regenerated. Ticket 45 ticked merged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YGQ3FjYgHS7jgMe6eLB7Z3
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -643,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -845,7 +845,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>gleif_last_update</t>
+          <t>gleif_legal_form</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -872,7 +872,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>gleif_legal_form</t>
+          <t>gleif_managing_lou</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -899,7 +899,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>gleif_managing_lou</t>
+          <t>gleif_registration_authority</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -926,7 +926,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>gleif_next_renewal</t>
+          <t>gleif_registration_authority_entity_id</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -953,7 +953,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>gleif_registration_authority</t>
+          <t>gleif_registration_status</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -980,7 +980,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>gleif_registration_authority_entity_id</t>
+          <t>gleif_validation_source</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>gleif_registration_status</t>
+          <t>jurisdiction</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1034,17 +1034,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>gleif_validation_source</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
+          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custodians.v1, sec.nport.registrant.v1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
+          <t>sec.submissions.company.v1</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1061,17 +1061,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>jurisdiction</t>
+          <t>sic</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
+          <t>sec.submissions.company.v1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
+          <t>sec.submissions.company.v1</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1088,12 +1088,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>state_of_incorporation</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>sec.submissions.company.v1, gleif.level1.v1, iapd.adv.filings.v1, iapd.adv.custodians.v1, sec.nport.registrant.v1</t>
+          <t>sec.submissions.company.v1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1107,87 +1107,6 @@
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/company.yaml defaults.sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>sic</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Kind default</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/company.yaml defaults.sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>sic_description</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Kind default</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/company.yaml defaults.sources</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>state_of_incorporation</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Kind default</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/company.yaml defaults.sources</t>
         </is>

</xml_diff>

<commit_message>
Ticket 09: P5 matches on the name and the city or postcode; P1 and P4 deleted
Operator, 2026-10-30 20:30 ET: "do not use p1 or p4, p5 can match on
postel code"; of the 4 flagged pairs P5 then links, "Link them
(Recommended)".

A cascade pass part may be a list of parts, any one agreeing enough, in
the census (cascade.agrees) and the Merge Stage re-check (Rust
addresses_agree). P5's measured entry: every new link over the whole SEC
population labelled, 251/251 the same entity, 159 adversarial, 0 different.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/merge/kinds/company.xlsx
+++ b/rules/merge/kinds/company.xlsx
@@ -1757,7 +1757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1980,12 +1980,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p1</t>
+          <t>sec-gleif-cascade-p5</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28.1</t>
+          <t>2026-10-30.1</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Pass P1: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, street, city, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city or postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p4</t>
+          <t>sec-gleif-cascade-p6</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Pass P4: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, postcode. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p5</t>
+          <t>sec-gleif-cascade-p7</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Pass P5: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country, city. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2106,32 +2106,28 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p6</t>
+          <t>iapd-adv-crd</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28.1</t>
+          <t>2026-10-09.1</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
+          <t>iapd.adv.filings.v1</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Pass P6: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the country. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>The record's CRD is the one a Company holds; and Exactly one Company holds that CRD, or none</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>mint</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -2148,32 +2144,28 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>sec-gleif-cascade-p7</t>
+          <t>iapd-adv-custodian-lei</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28.1</t>
+          <t>2026-10-09.1</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>gleif.level1.v1</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>sec.submissions.company.v1</t>
-        </is>
-      </c>
+          <t>iapd.adv.custodians.v1</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Pass P7: the names are equal, legal form kept (GLEIF's other names count), and, of what earlier passes left, exactly one SEC company and one GLEIF entity agree on the name alone. An address more than 25 entities share counts by its country only. Refused flags: none; and The GLEIF entity is GENERAL, ACTIVE, and not ANNULLED, DUPLICATE; and The SEC company is not already linked to another LEI</t>
+          <t>The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>mint</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -2190,7 +2182,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>iapd-adv-crd</t>
+          <t>iapd-adv-custodian-bd</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2200,13 +2192,13 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.filings.v1</t>
+          <t>iapd.adv.custodians.v1</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>The record's CRD is the one a Company holds; and Exactly one Company holds that CRD, or none</t>
+          <t>The record's BD_NUMBER is the one a Company holds; and Exactly one Company holds that BD_NUMBER, or none</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2228,109 +2220,33 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>iapd-adv-custodian-lei</t>
+          <t>gleif-issuer-lei</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09.1</t>
+          <t>2026-10-16.2</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>iapd.adv.custodians.v1</t>
+          <t>gleif.level1.v1</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
+          <t>The record has provenance.matching.nport_issuer; and The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>mint</t>
+          <t>wait</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>merge/kinds/company.yaml rules[11]</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>iapd-adv-custodian-bd</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09.1</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>iapd.adv.custodians.v1</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>The record's BD_NUMBER is the one a Company holds; and Exactly one Company holds that BD_NUMBER, or none</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>mint</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/company.yaml rules[12]</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>gleif-issuer-lei</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-16.2</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>gleif.level1.v1</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>The record has provenance.matching.nport_issuer; and The record's LEI is the one a Company holds; and Exactly one Company holds that LEI, or none</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>wait</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>merge/kinds/company.yaml rules[13]</t>
         </is>
       </c>
     </row>

</xml_diff>